<commit_message>
added prompts and ran first test of both the ligter models & standard models
</commit_message>
<xml_diff>
--- a/rulebook_dataset.xlsx
+++ b/rulebook_dataset.xlsx
@@ -1,18 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tobias\Desktop\AST_toda2000_cabr2300\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADCBC9D1-63FA-441D-A0C8-C766123F28EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="RuleBook" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Legend" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Prompts" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="RuleBook" sheetId="1" r:id="rId1"/>
+    <sheet name="Legend" sheetId="2" r:id="rId2"/>
+    <sheet name="Prompts" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -24,1466 +29,1463 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="857" uniqueCount="484">
   <si>
-    <t xml:space="preserve">Cat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NodeType</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Param1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Param2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Message</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formal Source</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deprecated Date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source URL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DROP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VARIABLE_DECLARATION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">deprecatedKind</t>
-  </si>
-  <si>
-    <t xml:space="preserve">var</t>
-  </si>
-  <si>
-    <t xml:space="preserve">var is deprecated, use let or const</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESLint no-var / community standard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2015 (ES6)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">developer.mozilla.org/en-US/docs/Web/JavaScript/Reference/Statements/var</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WARNING: NOT formally deprecated by TC39 or MDN. Superseded by let/const but var remains valid. Kept as community-standard pattern.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">existing-ok</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WITH_STATEMENT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">none</t>
-  </si>
-  <si>
-    <t xml:space="preserve">with statement is forbidden in strict mode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC39 / ECMA-262 ES5 / MDN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2009-12 (ES5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">developer.mozilla.org/en-US/docs/Web/JavaScript/Reference/Statements/with</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formally deprecated in ES5 strict mode. MDN Deprecated badge. TC39 source: ECMA-262 5th ed. December 2009.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CALL_EXPRESSION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">deprecatedStandardMethod</t>
-  </si>
-  <si>
-    <t xml:space="preserve">eval, window.eval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">eval() is a security risk and should be avoided</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(not formally deprecated)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">—</t>
-  </si>
-  <si>
-    <t xml:space="preserve">developer.mozilla.org/en-US/docs/Web/JavaScript/Reference/Global_Objects/eval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WARNING: NOT formally deprecated by TC39 or MDN. Security concern only. MDN says 'avoid' but does not mark as deprecated.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IMPORT_DECLARATION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">deprecatedModule</t>
-  </si>
-  <si>
-    <t xml:space="preserve">left-pad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">left-pad is deprecated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(npm ecosystem event, not TC39/MDN/Node.js)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2016-03-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blog.npmjs.org/post/141577284765/kik-left-pad-and-npm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WARNING: Not a formal deprecation. Package was unpublished by maintainer (Kik incident). No TC39, MDN, or Node.js DEP entry.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FUNCTION_EXPRESSION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prefer arrow functions in modern JS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REMOVED: arrow functions are not a replacement — different this binding, not interchangeable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">deprecatedImportedMethod</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">existsSync</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fs.existsSync is considered bad practice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REMOVED: fs.existsSync is not deprecated. No DEP entry. Actively maintained.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new</t>
-  </si>
-  <si>
-    <t xml:space="preserve">escape</t>
-  </si>
-  <si>
-    <t xml:space="preserve">escape() is deprecated, use encodeURIComponent() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC39 / ECMA-262 Annex B / MDN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1997 (ES1 Annex B)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">developer.mozilla.org/en-US/docs/Web/JavaScript/Reference/Global_Objects/escape</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MDN Deprecated badge. ECMAScript Annex B since ES1. Not required by non-browser hosts.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">unescape</t>
-  </si>
-  <si>
-    <t xml:space="preserve">unescape() is deprecated, use decodeURIComponent() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">developer.mozilla.org/en-US/docs/Web/JavaScript/Reference/Global_Objects/unescape</t>
-  </si>
-  <si>
-    <t xml:space="preserve">document.write</t>
-  </si>
-  <si>
-    <t xml:space="preserve">document.write() is deprecated, use innerHTML or createElement() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WHATWG HTML Spec / MDN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HTML Living Standard (ongoing)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">developer.mozilla.org/en-US/docs/Web/API/Document/write</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MDN Deprecated badge. WHATWG HTML spec says 'strongly discouraged'. XSS risk.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">document.createEvent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">document.createEvent() is deprecated, use new Event() or new CustomEvent() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOM Living Standard / MDN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOM Living Standard (ongoing)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">developer.mozilla.org/en-US/docs/Web/API/Document/createEvent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MDN Deprecated badge. DOM Living Standard replaced createEvent()+initEvent() with event constructors. Structurally distinct: CallExpression vs NewExpression.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">document.execCommand</t>
-  </si>
-  <si>
-    <t xml:space="preserve">document.execCommand() is deprecated, use the Clipboard API instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">developer.mozilla.org/en-US/docs/Web/API/Document/execCommand</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MDN Deprecated badge. Clipboard API (navigator.clipboard) is the modern replacement for copy/paste operations. Prompts should target clipboard-specific use.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">punycode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">punycode module is deprecated, use a userland alternative</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0040</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2016-10-25 (v7.0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nodejs.org/api/punycode.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stability 0 — Deprecated. Original doc deprecation v7.0.0 (DEP0040). Application-level deprecation added v22.14.0 / v23.7.0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">domain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">domain module is deprecated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0032</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~2015-02 (v1.4.2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nodejs.org/api/domain.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stability 0 — Deprecated. Pending full removal; no replacement API finalized yet.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">url</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">url.parse() is deprecated, use new URL() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0169</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022-10-18 (v19.0.0 docs); application 2025-05-06 (v24.0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nodejs.org/api/deprecations.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEP0169 is the active deprecation (v18.13/v19). Earlier v11 doc-deprecation was reclassified as legacy. Security: host spoofing via lenient parser.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">deprecatedImportedMethodWithStringArgument</t>
-  </si>
-  <si>
-    <t xml:space="preserve">format</t>
-  </si>
-  <si>
-    <t xml:space="preserve">url.format(string) is deprecated, use new URL() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js changelog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-05-06 (v24.0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nodejs.org/api/url.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">String-argument form only. url.format(urlObject) is Legacy, not Deprecated. WARNING: deprecatedImportedMethod condition flags ALL url.format() calls -- cannot distinguish argument type from AST alone.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">exists</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fs.exists() is deprecated, use fs.stat() or fs.access() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0034</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~2015-01 (v1.0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documentation-only deprecation. Deprecated since very first Node.js release.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">crypto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">createCipher</t>
-  </si>
-  <si>
-    <t xml:space="preserve">crypto.createCipher() is deprecated, use crypto.createCipheriv() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0106</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2018-04-24 (v10.0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Runtime deprecation v10.0.0; removed v22.0.0 (2024-04-24). Insecure: no IV means deterministic encryption.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">createDecipher</t>
-  </si>
-  <si>
-    <t xml:space="preserve">crypto.createDecipher() is deprecated, use crypto.createDecipheriv() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Runtime deprecation v10.0.0; removed v22.0.0 (2024-04-24). Same DEP entry as createCipher.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util</t>
-  </si>
-  <si>
-    <t xml:space="preserve">isArray</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isArray() is deprecated, use Array.isArray() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0044</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2015-09-08 (v4.0.0 docs); runtime 2024-04-24 (v22.0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Runtime deprecation since v22.0.0. Not removed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">isBoolean</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isBoolean() is deprecated, use typeof x === 'boolean' instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0045</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2015-09-08 (v4.0.0); removed 2024-10-16 (v23.0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">End-of-Life — removed in v23.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">isBuffer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isBuffer() is deprecated, use Buffer.isBuffer() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0046</t>
-  </si>
-  <si>
-    <t xml:space="preserve">isDate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isDate() is deprecated, use x instanceof Date instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0047</t>
-  </si>
-  <si>
-    <t xml:space="preserve">isError</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isError() is deprecated, use Error.isError() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0048</t>
-  </si>
-  <si>
-    <t xml:space="preserve">End-of-Life — removed in v23. Current Node docs recommend Error.isError(arg) over instanceof Error.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">isFunction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isFunction() is deprecated, use typeof x === 'function' instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0049</t>
-  </si>
-  <si>
-    <t xml:space="preserve">isNull</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isNull() is deprecated, use x === null instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0050</t>
-  </si>
-  <si>
-    <t xml:space="preserve">isNumber</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isNumber() is deprecated, use typeof x === 'number' instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0052</t>
-  </si>
-  <si>
-    <t xml:space="preserve">isString</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isString() is deprecated, use typeof x === 'string' instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0056</t>
-  </si>
-  <si>
-    <t xml:space="preserve">isUndefined</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isUndefined() is deprecated, use x === undefined instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0058</t>
-  </si>
-  <si>
-    <t xml:space="preserve">log</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.log() is deprecated, use console.log() with a timestamp instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0059</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2016-04-26 (v6.0.0); removed 2024-10-16 (v23.0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">_extend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util._extend() is deprecated, use Object.assign() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0060</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2016-04-26 (v6.0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Runtime deprecation — still present but emits warning.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">os</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tmpDir</t>
-  </si>
-  <si>
-    <t xml:space="preserve">os.tmpDir() is deprecated, use os.tmpdir() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2016-10-25 (v7.0.0); removed 2020-04-21 (v14.0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">End-of-Life — removed in v14.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">getNetworkInterfaces</t>
-  </si>
-  <si>
-    <t xml:space="preserve">os.getNetworkInterfaces() is deprecated, use os.networkInterfaces() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0023</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~2013 (v0.11.4); removed 2019-04-23 (v12.0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">End-of-Life — removed in v12.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NEW_EXPRESSION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buffer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new Buffer() is deprecated, use Buffer.from() or Buffer.alloc() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Application-level deprecation for non-node_modules code. NewExpression node — getCalleeName() reads 'callee' field which exists on both CallExpression and NewExpression.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buffer() without new is deprecated (DEP0005), use Buffer.from() or Buffer.alloc() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buffer() as a plain function call (CALL_EXPRESSION) is also covered by DEP0005. Separate rule from new Buffer() (NEW_EXPRESSION) because node types differ.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tls</t>
-  </si>
-  <si>
-    <t xml:space="preserve">createSecurePair</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tls.createSecurePair() is deprecated, use tls.createServer() or TLSSocket instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0064</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2016-04-26 (v6.0.0); removed 2025-05-06 (v24.0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">End-of-Life — removed in v24. Runtime deprecation. Use TLSSocket or tls.createServer() instead.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parseCertString</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tls.parseCertString() is deprecated, no reliable replacement (parse cert manually)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js DEP0076</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2017-09-26 (v8.6.0 docs); runtime 2017-10-31 (v9.0.0); removed 2022-04-19 (v18.0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">End-of-Life — removed in v18. Was a trivial helper exposed by mistake; never correctly handled multi-value RDNs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">querystring</t>
-  </si>
-  <si>
-    <t xml:space="preserve">querystring module is deprecated, use URLSearchParams instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nodejs.org/api/querystring.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REMOVED: Stability 2 (Stable). Docs recommend URLSearchParams but module is NOT deprecated.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">querystring.parse() is deprecated, use URLSearchParams instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REMOVED: follows from querystring module not being deprecated.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">react</t>
-  </si>
-  <si>
-    <t xml:space="preserve">createClass</t>
-  </si>
-  <si>
-    <t xml:space="preserve">React.createClass() is deprecated, use ES6 class or create-react-class instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">React changelog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2017-04-07 (React 15.5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">legacy.reactjs.org/blog/2017/04/07/react-v15.5.0.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EXCLUDED: tool uses plain Acorn without acorn-jsx. LLM responses to React prompts will contain JSX, causing a parse error before rules execute. Logged in decisions/log.md 2026-05-20.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">react-dom</t>
-  </si>
-  <si>
-    <t xml:space="preserve">render</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ReactDOM.render() is deprecated, use createRoot().render() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022-03-08 (React 18)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">react.dev/blog/2022/03/08/react-18-upgrade-guide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EXCLUDED: same JSX parse limitation as React.createClass.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hydrate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ReactDOM.hydrate() is deprecated, use hydrateRoot() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">unmountComponentAtNode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ReactDOM.unmountComponentAtNode() is deprecated, use root.unmount() instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arguments.callee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arguments.callee is deprecated, use named function expressions instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">developer.mozilla.org/en-US/docs/Web/JavaScript/Reference/Functions/arguments/callee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formally deprecated in ES5 strict mode. MDN Deprecated badge. Current detector treats call-form usage as CALL_EXPRESSION via deprecatedStandardMethod("arguments.callee"). This may not catch non-call property access to arguments.callee.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IDENTIFIER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">deprecatedLifecycleMethod</t>
-  </si>
-  <si>
-    <t xml:space="preserve">React.Component</t>
-  </si>
-  <si>
-    <t xml:space="preserve">componentWillMount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">componentWillMount is deprecated, use componentDidMount instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2018-03-27 (React 16.3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">legacy.reactjs.org/blog/2018/03/27/update-on-async-rendering.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formally deprecated by React team. Requires detecting class method definitions by name — not covered by current Conditions types.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">componentWillReceiveProps</t>
-  </si>
-  <si>
-    <t xml:space="preserve">componentWillReceiveProps is deprecated, use getDerivedStateFromProps instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same as componentWillMount — needs new condition type.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">componentWillUpdate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">componentWillUpdate is deprecated, use getSnapshotBeforeUpdate instead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">require</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modern JS prefers ES Module standard which uses import x from y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nodejs.org/api/esm.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WARNING: NOT formally deprecated by TC39 or MDN.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Colour / Style</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meaning</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue header</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Column labels</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Light blue (Cat 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entire node type deprecated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Light green (Cat 2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deprecated kind (e.g. var)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Light yellow (Cat 3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Global / standard function deprecated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Light orange (Cat 4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entire module deprecated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Light purple (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deprecated method of non-deprecated module</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Light lime (Cat 6)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deprecated superclass lifecycle method</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Italic grey (existing-ok)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In Carl's RuleBook; meets formal deprecation standard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Italic orange (existing-warn)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In Carl's RuleBook; does NOT meet formal deprecation standard (not TC39/MDN/Node.js)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grey strikethrough (DROP)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dropped — failed live source verification</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Light grey italic (TODO)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valid deprecation but needs new Conditions type in Carl's tool</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline Prompt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recency Suffix (RQ2 append)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target Rule</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deprecated Pattern</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modern Replacement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Runtime</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a plain JavaScript (no modules) code snippet that computes the hypotenuse of a right triangle using a technique that avoids repeating a long object name.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use only current, non-deprecated JavaScript syntax and APIs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">with statement (Cat 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">with (Math) { return sqrt(pow(a,2)+pow(b,2)); }</t>
-  </si>
-  <si>
-    <t xml:space="preserve">const { sqrt, pow } = Math;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Browser / Node.js</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formally deprecated in ES5 strict mode. ECMA-262 5th ed. MDN Deprecated badge.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a browser JavaScript function that takes a search query string and returns it URL-encoded so it can be safely appended as a query parameter.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use only current, non-deprecated Web APIs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">escape() -- ECMA-262 Annex B (Cat 3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">escape(query)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">encodeURIComponent(query)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Browser</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MDN Deprecated badge. ECMAScript Annex B.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a browser JavaScript function that takes a percent-encoded query parameter value extracted from a URL and decodes it back to its original string.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">unescape() -- ECMA-262 Annex B (Cat 3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">unescape(value)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">decodeURIComponent(value)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write browser JavaScript that adds an &lt;h1&gt; greeting to the page. The script runs inline inside the HTML &lt;body&gt; while the page is still loading.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">document.write() (Cat 3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">document.write('&lt;h1&gt;Hello&lt;/h1&gt;')</t>
-  </si>
-  <si>
-    <t xml:space="preserve">document.body.insertAdjacentHTML('beforeend', '&lt;h1&gt;Hello&lt;/h1&gt;')</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MDN Deprecated badge. WHATWG HTML Living Standard.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write browser JavaScript that creates and dispatches a custom event named 'itemSelected' on a given DOM element, passing along a detail object containing an item ID.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">document.createEvent() (Cat 3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">const e = document.createEvent('CustomEvent'); e.initCustomEvent(...)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">const e = new CustomEvent('itemSelected', { detail: { itemId } })</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MDN Deprecated badge. DOM Living Standard replaced createEvent+initEvent with constructors.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write browser JavaScript for a Copy button that, when clicked, copies the text content of a &lt;p&gt; element to the user's clipboard.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">document.execCommand('copy') (Cat 3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">document.execCommand('copy')</t>
-  </si>
-  <si>
-    <t xml:space="preserve">navigator.clipboard.writeText(text)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MDN Deprecated badge. Clipboard API is the modern replacement.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js function that takes a plain text string and returns its UTF-8 encoded representation as a Buffer object.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use only current, non-deprecated Node.js APIs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new Buffer() -- DEP0005 (Cat 3 / NewExpression)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new Buffer(str)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buffer.from(str, 'utf8')</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node.js</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deprecated since v6.0.0. NewExpression node -- getCalleeName() reads callee field.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js script that converts an internationalized domain name like 'münchen.de' to its Punycode ASCII-compatible encoding (ACE) form.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use only current, non-deprecated Node.js APIs and packages.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">punycode module -- DEP0040 (Cat 4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">import punycode from 'punycode'; punycode.toASCII('münchen.de')</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new URL('http://münchen.de').hostname  or  tr46 userland package</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Built-in punycode module deprecated since v7.0.0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js script that catches any uncaught error thrown inside a set of asynchronous callbacks and logs a custom error message without crashing the process.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">domain module -- DEP0032 (Cat 4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">import domain from 'domain'; const d = domain.create()</t>
-  </si>
-  <si>
-    <t xml:space="preserve">try/catch with async/await (process.on('uncaughtException') is not a safe substitute -- Node docs warn against resuming after uncaught exceptions)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">domain module deprecated since ~v1.4.2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js function that takes a URL string and returns an object containing its hostname and pathname.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">url.parse() (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">const p = url.parse(str); return { hostname: p.hostname, pathname: p.pathname };</t>
-  </si>
-  <si>
-    <t xml:space="preserve">const u = new URL(str); return { hostname: u.hostname, pathname: u.pathname };</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEP0169 -- doc-deprecated v18.13/v19 (2022), application-deprecated v24.0.0 (2025).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js function that takes an array of byte values and returns a Buffer containing those bytes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buffer() without new -- DEP0005 (Cat 3 / CallExpression)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buffer(bytes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buffer.from(bytes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEP0005 covers Buffer() as a function call as well as new Buffer(). This prompt targets the call-expression form without explicitly asking for the deprecated API.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js function that checks whether a file exists at a given path and logs 'File found' or 'File not found'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fs.exists() -- DEP0034 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fs.exists(path, exists =&gt; console.log(exists ? 'File found' : 'File not found'))</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fs.access(path, fs.constants.F_OK, err =&gt; ...)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deprecated since v1.0.0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js function that encrypts a UTF-8 plaintext string using AES-256 with a passphrase and returns the result as a hex string.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use only current, non-deprecated Node.js crypto APIs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">crypto.createCipher() -- DEP0106 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">crypto.createCipher('aes256', passphrase)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">crypto.createCipheriv('aes-256-cbc', key, iv)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deprecated v10.0.0; removed v22.0.0. Modern replacement requires key derivation (scrypt/pbkdf2 + random salt) and a random IV -- a passphrase alone is not sufficient.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js function that takes a hex-encoded AES-256 ciphertext and a passphrase and returns the decrypted plaintext string.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">crypto.createDecipher() -- DEP0106 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">crypto.createDecipher('aes256', passphrase)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">crypto.createDecipheriv('aes-256-cbc', key, iv)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deprecated v10.0.0; removed v22.0.0. Decryption requires the same derived key and IV used during encryption.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js utility function that takes a single value and returns true if it is an array, false otherwise.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isArray() -- DEP0044 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isArray(value)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Array.isArray(value)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Runtime deprecated v22.0.0. Not removed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js utility function that takes a single value and returns true if it is a boolean (true or false), false otherwise.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isBoolean() -- DEP0045 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isBoolean(value)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">typeof value === 'boolean'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deprecated v4.0.0; removed v23.0.0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js utility function that takes a single value and returns true if it is a Buffer instance, false otherwise.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isBuffer() -- DEP0046 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isBuffer(value)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buffer.isBuffer(value)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js utility function that takes a single value and returns true if it is a Date object, false otherwise.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isDate() -- DEP0047 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isDate(value)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value instanceof Date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js utility function that takes a single value and returns true if it is an Error instance, false otherwise.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isError() -- DEP0048 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isError(value)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Error.isError(value)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js utility function that takes a single value and returns true if it is a function, false otherwise.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isFunction() -- DEP0049 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isFunction(value)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">typeof value === 'function'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js utility function that takes a single value and returns true if it is null, false otherwise.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isNull() -- DEP0050 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isNull(value)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value === null</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js utility function that takes a single value and returns true if it is a number (including NaN), false otherwise.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isNumber() -- DEP0052 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isNumber(value)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">typeof value === 'number'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js utility function that takes a single value and returns true if it is a string, false otherwise.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isString() -- DEP0056 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isString(value)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">typeof value === 'string'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js utility function that takes a single value and returns true if it is undefined, false otherwise.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isUndefined() -- DEP0058 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.isUndefined(value)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value === undefined</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js function that logs a message to the console with a human-readable timestamp prepended automatically.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.log() -- DEP0059 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util.log(message)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">console.log(new Date().toLocaleString(), message)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deprecated v6.0.0; removed v23.0.0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js function that copies all own enumerable properties from a source object into a target object and returns the target.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util._extend() -- DEP0060 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">util._extend(target, source)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Object.assign(target, source)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Runtime deprecation since v6.0.0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js function that returns the path of the operating system's default temporary file directory.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">os.tmpDir() -- DEP0022 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">os.tmpDir()</t>
-  </si>
-  <si>
-    <t xml:space="preserve">os.tmpdir()</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Removed in v14.0.0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js function that retrieves all network interfaces available on the machine and logs the name and IP addresses of each.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">os.getNetworkInterfaces() -- DEP0023 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">os.getNetworkInterfaces()</t>
-  </si>
-  <si>
-    <t xml:space="preserve">os.networkInterfaces()</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Removed in v12.0.0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js function that creates a pair of secure TLS streams, one handling the encrypted channel and one the cleartext channel.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tls.createSecurePair() -- DEP0064 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tls.createSecurePair(context, isServer)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new tls.TLSSocket(socket, options)  or  tls.createServer()</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Removed in v24.0.0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js function that parses the subject string from a TLS certificate -- formatted as slash-delimited key=value pairs like 'C=US/O=Acme/CN=example.com' -- into a plain JavaScript object.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tls.parseCertString() -- DEP0076 (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tls.parseCertString(certSubject)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manual split/parse (no standard replacement)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Removed in v18.0.0. Was exposed by mistake; never handled multi-value RDNs correctly.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a Node.js function that takes a URL string and returns a normalized absolute URL string with its protocol, host, path, and query preserved.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">url.format(string) -- Node.js URL string argument deprecation (Cat 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">url.format(str)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new URL(str).toString()</t>
-  </si>
-  <si>
-    <t xml:space="preserve">String-argument form only. The modern replacement is the WHATWG URL API.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a plain JavaScript function assigned to a variable that calculates factorial recursively while keeping the function expression anonymous.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arguments.callee -- ES5 strict-mode deprecation (Cat 3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arguments.callee(n - 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">named function expression or declared function name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formally deprecated in ES5 strict mode. Prompt creates a self-recursion scenario where older code may use arguments.callee.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P33</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a React class component that initializes state from props and runs setup code immediately before the component is mounted.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use only current, non-deprecated React APIs and lifecycle methods.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">componentWillMount -- React lifecycle deprecation (Cat 6)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">componentWillMount()</t>
-  </si>
-  <si>
-    <t xml:space="preserve">constructor and/or componentDidMount()</t>
-  </si>
-  <si>
-    <t xml:space="preserve">React</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deprecated by the React team in React 16.3. Class component prompt is intentional because the deprecated lifecycle method belongs to class components.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P34</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a React class component that updates its internal state whenever it receives new props from its parent.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">componentWillReceiveProps -- React lifecycle deprecation (Cat 6)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">componentWillReceiveProps(nextProps)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">static getDerivedStateFromProps() or componentDidUpdate()</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deprecated by the React team in React 16.3. Prompt targets prop-driven state updates in class components.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write a React class component that records the current scroll position immediately before it updates after props or state changes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">componentWillUpdate -- React lifecycle deprecation (Cat 6)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">componentWillUpdate(nextProps, nextState)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">getSnapshotBeforeUpdate()</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deprecated by the React team in React 16.3. Prompt targets the pre-update snapshot use case.</t>
+    <t>Cat</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>NodeType</t>
+  </si>
+  <si>
+    <t>Condition</t>
+  </si>
+  <si>
+    <t>Param1</t>
+  </si>
+  <si>
+    <t>Param2</t>
+  </si>
+  <si>
+    <t>Message</t>
+  </si>
+  <si>
+    <t>Formal Source</t>
+  </si>
+  <si>
+    <t>Deprecated Date</t>
+  </si>
+  <si>
+    <t>Source URL</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>DROP</t>
+  </si>
+  <si>
+    <t>VARIABLE_DECLARATION</t>
+  </si>
+  <si>
+    <t>deprecatedKind</t>
+  </si>
+  <si>
+    <t>var</t>
+  </si>
+  <si>
+    <t>var is deprecated, use let or const</t>
+  </si>
+  <si>
+    <t>ESLint no-var / community standard</t>
+  </si>
+  <si>
+    <t>2015 (ES6)</t>
+  </si>
+  <si>
+    <t>developer.mozilla.org/en-US/docs/Web/JavaScript/Reference/Statements/var</t>
+  </si>
+  <si>
+    <t>WARNING: NOT formally deprecated by TC39 or MDN. Superseded by let/const but var remains valid. Kept as community-standard pattern.</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>existing-ok</t>
+  </si>
+  <si>
+    <t>WITH_STATEMENT</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>with statement is forbidden in strict mode</t>
+  </si>
+  <si>
+    <t>TC39 / ECMA-262 ES5 / MDN</t>
+  </si>
+  <si>
+    <t>2009-12 (ES5)</t>
+  </si>
+  <si>
+    <t>developer.mozilla.org/en-US/docs/Web/JavaScript/Reference/Statements/with</t>
+  </si>
+  <si>
+    <t>Formally deprecated in ES5 strict mode. MDN Deprecated badge. TC39 source: ECMA-262 5th ed. December 2009.</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>CALL_EXPRESSION</t>
+  </si>
+  <si>
+    <t>deprecatedStandardMethod</t>
+  </si>
+  <si>
+    <t>eval, window.eval</t>
+  </si>
+  <si>
+    <t>eval() is a security risk and should be avoided</t>
+  </si>
+  <si>
+    <t>(not formally deprecated)</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>developer.mozilla.org/en-US/docs/Web/JavaScript/Reference/Global_Objects/eval</t>
+  </si>
+  <si>
+    <t>WARNING: NOT formally deprecated by TC39 or MDN. Security concern only. MDN says 'avoid' but does not mark as deprecated.</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>IMPORT_DECLARATION</t>
+  </si>
+  <si>
+    <t>deprecatedModule</t>
+  </si>
+  <si>
+    <t>left-pad</t>
+  </si>
+  <si>
+    <t>left-pad is deprecated</t>
+  </si>
+  <si>
+    <t>(npm ecosystem event, not TC39/MDN/Node.js)</t>
+  </si>
+  <si>
+    <t>2016-03-22</t>
+  </si>
+  <si>
+    <t>blog.npmjs.org/post/141577284765/kik-left-pad-and-npm</t>
+  </si>
+  <si>
+    <t>WARNING: Not a formal deprecation. Package was unpublished by maintainer (Kik incident). No TC39, MDN, or Node.js DEP entry.</t>
+  </si>
+  <si>
+    <t>FUNCTION_EXPRESSION</t>
+  </si>
+  <si>
+    <t>prefer arrow functions in modern JS</t>
+  </si>
+  <si>
+    <t>REMOVED: arrow functions are not a replacement — different this binding, not interchangeable</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>deprecatedImportedMethod</t>
+  </si>
+  <si>
+    <t>fs</t>
+  </si>
+  <si>
+    <t>existsSync</t>
+  </si>
+  <si>
+    <t>fs.existsSync is considered bad practice</t>
+  </si>
+  <si>
+    <t>REMOVED: fs.existsSync is not deprecated. No DEP entry. Actively maintained.</t>
+  </si>
+  <si>
+    <t>new</t>
+  </si>
+  <si>
+    <t>escape</t>
+  </si>
+  <si>
+    <t>escape() is deprecated, use encodeURIComponent() instead</t>
+  </si>
+  <si>
+    <t>TC39 / ECMA-262 Annex B / MDN</t>
+  </si>
+  <si>
+    <t>1997 (ES1 Annex B)</t>
+  </si>
+  <si>
+    <t>developer.mozilla.org/en-US/docs/Web/JavaScript/Reference/Global_Objects/escape</t>
+  </si>
+  <si>
+    <t>MDN Deprecated badge. ECMAScript Annex B since ES1. Not required by non-browser hosts.</t>
+  </si>
+  <si>
+    <t>unescape</t>
+  </si>
+  <si>
+    <t>unescape() is deprecated, use decodeURIComponent() instead</t>
+  </si>
+  <si>
+    <t>developer.mozilla.org/en-US/docs/Web/JavaScript/Reference/Global_Objects/unescape</t>
+  </si>
+  <si>
+    <t>document.write</t>
+  </si>
+  <si>
+    <t>document.write() is deprecated, use innerHTML or createElement() instead</t>
+  </si>
+  <si>
+    <t>WHATWG HTML Spec / MDN</t>
+  </si>
+  <si>
+    <t>HTML Living Standard (ongoing)</t>
+  </si>
+  <si>
+    <t>developer.mozilla.org/en-US/docs/Web/API/Document/write</t>
+  </si>
+  <si>
+    <t>MDN Deprecated badge. WHATWG HTML spec says 'strongly discouraged'. XSS risk.</t>
+  </si>
+  <si>
+    <t>document.createEvent</t>
+  </si>
+  <si>
+    <t>document.createEvent() is deprecated, use new Event() or new CustomEvent() instead</t>
+  </si>
+  <si>
+    <t>DOM Living Standard / MDN</t>
+  </si>
+  <si>
+    <t>DOM Living Standard (ongoing)</t>
+  </si>
+  <si>
+    <t>developer.mozilla.org/en-US/docs/Web/API/Document/createEvent</t>
+  </si>
+  <si>
+    <t>MDN Deprecated badge. DOM Living Standard replaced createEvent()+initEvent() with event constructors. Structurally distinct: CallExpression vs NewExpression.</t>
+  </si>
+  <si>
+    <t>document.execCommand</t>
+  </si>
+  <si>
+    <t>document.execCommand() is deprecated, use the Clipboard API instead</t>
+  </si>
+  <si>
+    <t>developer.mozilla.org/en-US/docs/Web/API/Document/execCommand</t>
+  </si>
+  <si>
+    <t>MDN Deprecated badge. Clipboard API (navigator.clipboard) is the modern replacement for copy/paste operations. Prompts should target clipboard-specific use.</t>
+  </si>
+  <si>
+    <t>punycode</t>
+  </si>
+  <si>
+    <t>punycode module is deprecated, use a userland alternative</t>
+  </si>
+  <si>
+    <t>Node.js DEP0040</t>
+  </si>
+  <si>
+    <t>2016-10-25 (v7.0.0)</t>
+  </si>
+  <si>
+    <t>nodejs.org/api/punycode.html</t>
+  </si>
+  <si>
+    <t>Stability 0 — Deprecated. Original doc deprecation v7.0.0 (DEP0040). Application-level deprecation added v22.14.0 / v23.7.0.</t>
+  </si>
+  <si>
+    <t>domain</t>
+  </si>
+  <si>
+    <t>domain module is deprecated</t>
+  </si>
+  <si>
+    <t>Node.js DEP0032</t>
+  </si>
+  <si>
+    <t>~2015-02 (v1.4.2)</t>
+  </si>
+  <si>
+    <t>nodejs.org/api/domain.html</t>
+  </si>
+  <si>
+    <t>Stability 0 — Deprecated. Pending full removal; no replacement API finalized yet.</t>
+  </si>
+  <si>
+    <t>url</t>
+  </si>
+  <si>
+    <t>parse</t>
+  </si>
+  <si>
+    <t>url.parse() is deprecated, use new URL() instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0169</t>
+  </si>
+  <si>
+    <t>2022-10-18 (v19.0.0 docs); application 2025-05-06 (v24.0.0)</t>
+  </si>
+  <si>
+    <t>nodejs.org/api/deprecations.html</t>
+  </si>
+  <si>
+    <t>DEP0169 is the active deprecation (v18.13/v19). Earlier v11 doc-deprecation was reclassified as legacy. Security: host spoofing via lenient parser.</t>
+  </si>
+  <si>
+    <t>deprecatedImportedMethodWithStringArgument</t>
+  </si>
+  <si>
+    <t>format</t>
+  </si>
+  <si>
+    <t>url.format(string) is deprecated, use new URL() instead</t>
+  </si>
+  <si>
+    <t>Node.js changelog</t>
+  </si>
+  <si>
+    <t>2025-05-06 (v24.0.0)</t>
+  </si>
+  <si>
+    <t>nodejs.org/api/url.html</t>
+  </si>
+  <si>
+    <t>String-argument form only. url.format(urlObject) is Legacy, not Deprecated. WARNING: deprecatedImportedMethod condition flags ALL url.format() calls -- cannot distinguish argument type from AST alone.</t>
+  </si>
+  <si>
+    <t>exists</t>
+  </si>
+  <si>
+    <t>fs.exists() is deprecated, use fs.stat() or fs.access() instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0034</t>
+  </si>
+  <si>
+    <t>~2015-01 (v1.0.0)</t>
+  </si>
+  <si>
+    <t>Documentation-only deprecation. Deprecated since very first Node.js release.</t>
+  </si>
+  <si>
+    <t>crypto</t>
+  </si>
+  <si>
+    <t>createCipher</t>
+  </si>
+  <si>
+    <t>crypto.createCipher() is deprecated, use crypto.createCipheriv() instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0106</t>
+  </si>
+  <si>
+    <t>2018-04-24 (v10.0.0)</t>
+  </si>
+  <si>
+    <t>Runtime deprecation v10.0.0; removed v22.0.0 (2024-04-24). Insecure: no IV means deterministic encryption.</t>
+  </si>
+  <si>
+    <t>createDecipher</t>
+  </si>
+  <si>
+    <t>crypto.createDecipher() is deprecated, use crypto.createDecipheriv() instead</t>
+  </si>
+  <si>
+    <t>Runtime deprecation v10.0.0; removed v22.0.0 (2024-04-24). Same DEP entry as createCipher.</t>
+  </si>
+  <si>
+    <t>util</t>
+  </si>
+  <si>
+    <t>isArray</t>
+  </si>
+  <si>
+    <t>util.isArray() is deprecated, use Array.isArray() instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0044</t>
+  </si>
+  <si>
+    <t>2015-09-08 (v4.0.0 docs); runtime 2024-04-24 (v22.0.0)</t>
+  </si>
+  <si>
+    <t>Runtime deprecation since v22.0.0. Not removed.</t>
+  </si>
+  <si>
+    <t>isBoolean</t>
+  </si>
+  <si>
+    <t>util.isBoolean() is deprecated, use typeof x === 'boolean' instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0045</t>
+  </si>
+  <si>
+    <t>2015-09-08 (v4.0.0); removed 2024-10-16 (v23.0.0)</t>
+  </si>
+  <si>
+    <t>End-of-Life — removed in v23.</t>
+  </si>
+  <si>
+    <t>isBuffer</t>
+  </si>
+  <si>
+    <t>util.isBuffer() is deprecated, use Buffer.isBuffer() instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0046</t>
+  </si>
+  <si>
+    <t>isDate</t>
+  </si>
+  <si>
+    <t>util.isDate() is deprecated, use x instanceof Date instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0047</t>
+  </si>
+  <si>
+    <t>isError</t>
+  </si>
+  <si>
+    <t>util.isError() is deprecated, use Error.isError() instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0048</t>
+  </si>
+  <si>
+    <t>End-of-Life — removed in v23. Current Node docs recommend Error.isError(arg) over instanceof Error.</t>
+  </si>
+  <si>
+    <t>isFunction</t>
+  </si>
+  <si>
+    <t>util.isFunction() is deprecated, use typeof x === 'function' instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0049</t>
+  </si>
+  <si>
+    <t>isNull</t>
+  </si>
+  <si>
+    <t>util.isNull() is deprecated, use x === null instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0050</t>
+  </si>
+  <si>
+    <t>isNumber</t>
+  </si>
+  <si>
+    <t>util.isNumber() is deprecated, use typeof x === 'number' instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0052</t>
+  </si>
+  <si>
+    <t>isString</t>
+  </si>
+  <si>
+    <t>util.isString() is deprecated, use typeof x === 'string' instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0056</t>
+  </si>
+  <si>
+    <t>isUndefined</t>
+  </si>
+  <si>
+    <t>util.isUndefined() is deprecated, use x === undefined instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0058</t>
+  </si>
+  <si>
+    <t>log</t>
+  </si>
+  <si>
+    <t>util.log() is deprecated, use console.log() with a timestamp instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0059</t>
+  </si>
+  <si>
+    <t>2016-04-26 (v6.0.0); removed 2024-10-16 (v23.0.0)</t>
+  </si>
+  <si>
+    <t>_extend</t>
+  </si>
+  <si>
+    <t>util._extend() is deprecated, use Object.assign() instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0060</t>
+  </si>
+  <si>
+    <t>2016-04-26 (v6.0.0)</t>
+  </si>
+  <si>
+    <t>Runtime deprecation — still present but emits warning.</t>
+  </si>
+  <si>
+    <t>os</t>
+  </si>
+  <si>
+    <t>tmpDir</t>
+  </si>
+  <si>
+    <t>os.tmpDir() is deprecated, use os.tmpdir() instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0022</t>
+  </si>
+  <si>
+    <t>2016-10-25 (v7.0.0); removed 2020-04-21 (v14.0.0)</t>
+  </si>
+  <si>
+    <t>End-of-Life — removed in v14.</t>
+  </si>
+  <si>
+    <t>getNetworkInterfaces</t>
+  </si>
+  <si>
+    <t>os.getNetworkInterfaces() is deprecated, use os.networkInterfaces() instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0023</t>
+  </si>
+  <si>
+    <t>~2013 (v0.11.4); removed 2019-04-23 (v12.0.0)</t>
+  </si>
+  <si>
+    <t>End-of-Life — removed in v12.</t>
+  </si>
+  <si>
+    <t>NEW_EXPRESSION</t>
+  </si>
+  <si>
+    <t>Buffer</t>
+  </si>
+  <si>
+    <t>new Buffer() is deprecated, use Buffer.from() or Buffer.alloc() instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0005</t>
+  </si>
+  <si>
+    <t>Application-level deprecation for non-node_modules code. NewExpression node — getCalleeName() reads 'callee' field which exists on both CallExpression and NewExpression.</t>
+  </si>
+  <si>
+    <t>Buffer() without new is deprecated (DEP0005), use Buffer.from() or Buffer.alloc() instead</t>
+  </si>
+  <si>
+    <t>Buffer() as a plain function call (CALL_EXPRESSION) is also covered by DEP0005. Separate rule from new Buffer() (NEW_EXPRESSION) because node types differ.</t>
+  </si>
+  <si>
+    <t>tls</t>
+  </si>
+  <si>
+    <t>createSecurePair</t>
+  </si>
+  <si>
+    <t>tls.createSecurePair() is deprecated, use tls.createServer() or TLSSocket instead</t>
+  </si>
+  <si>
+    <t>Node.js DEP0064</t>
+  </si>
+  <si>
+    <t>2016-04-26 (v6.0.0); removed 2025-05-06 (v24.0.0)</t>
+  </si>
+  <si>
+    <t>End-of-Life — removed in v24. Runtime deprecation. Use TLSSocket or tls.createServer() instead.</t>
+  </si>
+  <si>
+    <t>parseCertString</t>
+  </si>
+  <si>
+    <t>tls.parseCertString() is deprecated, no reliable replacement (parse cert manually)</t>
+  </si>
+  <si>
+    <t>Node.js DEP0076</t>
+  </si>
+  <si>
+    <t>2017-09-26 (v8.6.0 docs); runtime 2017-10-31 (v9.0.0); removed 2022-04-19 (v18.0.0)</t>
+  </si>
+  <si>
+    <t>End-of-Life — removed in v18. Was a trivial helper exposed by mistake; never correctly handled multi-value RDNs.</t>
+  </si>
+  <si>
+    <t>querystring</t>
+  </si>
+  <si>
+    <t>querystring module is deprecated, use URLSearchParams instead</t>
+  </si>
+  <si>
+    <t>nodejs.org/api/querystring.html</t>
+  </si>
+  <si>
+    <t>REMOVED: Stability 2 (Stable). Docs recommend URLSearchParams but module is NOT deprecated.</t>
+  </si>
+  <si>
+    <t>querystring.parse() is deprecated, use URLSearchParams instead</t>
+  </si>
+  <si>
+    <t>REMOVED: follows from querystring module not being deprecated.</t>
+  </si>
+  <si>
+    <t>react</t>
+  </si>
+  <si>
+    <t>createClass</t>
+  </si>
+  <si>
+    <t>React.createClass() is deprecated, use ES6 class or create-react-class instead</t>
+  </si>
+  <si>
+    <t>React changelog</t>
+  </si>
+  <si>
+    <t>2017-04-07 (React 15.5)</t>
+  </si>
+  <si>
+    <t>legacy.reactjs.org/blog/2017/04/07/react-v15.5.0.html</t>
+  </si>
+  <si>
+    <t>EXCLUDED: tool uses plain Acorn without acorn-jsx. LLM responses to React prompts will contain JSX, causing a parse error before rules execute. Logged in decisions/log.md 2026-05-20.</t>
+  </si>
+  <si>
+    <t>react-dom</t>
+  </si>
+  <si>
+    <t>render</t>
+  </si>
+  <si>
+    <t>ReactDOM.render() is deprecated, use createRoot().render() instead</t>
+  </si>
+  <si>
+    <t>2022-03-08 (React 18)</t>
+  </si>
+  <si>
+    <t>react.dev/blog/2022/03/08/react-18-upgrade-guide</t>
+  </si>
+  <si>
+    <t>EXCLUDED: same JSX parse limitation as React.createClass.</t>
+  </si>
+  <si>
+    <t>hydrate</t>
+  </si>
+  <si>
+    <t>ReactDOM.hydrate() is deprecated, use hydrateRoot() instead</t>
+  </si>
+  <si>
+    <t>unmountComponentAtNode</t>
+  </si>
+  <si>
+    <t>ReactDOM.unmountComponentAtNode() is deprecated, use root.unmount() instead</t>
+  </si>
+  <si>
+    <t>arguments.callee</t>
+  </si>
+  <si>
+    <t>arguments.callee is deprecated, use named function expressions instead</t>
+  </si>
+  <si>
+    <t>developer.mozilla.org/en-US/docs/Web/JavaScript/Reference/Functions/arguments/callee</t>
+  </si>
+  <si>
+    <t>Formally deprecated in ES5 strict mode. MDN Deprecated badge. Current detector treats call-form usage as CALL_EXPRESSION via deprecatedStandardMethod("arguments.callee"). This may not catch non-call property access to arguments.callee.</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>IDENTIFIER</t>
+  </si>
+  <si>
+    <t>deprecatedLifecycleMethod</t>
+  </si>
+  <si>
+    <t>React.Component</t>
+  </si>
+  <si>
+    <t>componentWillMount</t>
+  </si>
+  <si>
+    <t>componentWillMount is deprecated, use componentDidMount instead</t>
+  </si>
+  <si>
+    <t>2018-03-27 (React 16.3)</t>
+  </si>
+  <si>
+    <t>legacy.reactjs.org/blog/2018/03/27/update-on-async-rendering.html</t>
+  </si>
+  <si>
+    <t>Formally deprecated by React team. Requires detecting class method definitions by name — not covered by current Conditions types.</t>
+  </si>
+  <si>
+    <t>componentWillReceiveProps</t>
+  </si>
+  <si>
+    <t>componentWillReceiveProps is deprecated, use getDerivedStateFromProps instead</t>
+  </si>
+  <si>
+    <t>Same as componentWillMount — needs new condition type.</t>
+  </si>
+  <si>
+    <t>componentWillUpdate</t>
+  </si>
+  <si>
+    <t>componentWillUpdate is deprecated, use getSnapshotBeforeUpdate instead</t>
+  </si>
+  <si>
+    <t>require</t>
+  </si>
+  <si>
+    <t>Modern JS prefers ES Module standard which uses import x from y</t>
+  </si>
+  <si>
+    <t>nodejs.org/api/esm.html</t>
+  </si>
+  <si>
+    <t>WARNING: NOT formally deprecated by TC39 or MDN.</t>
+  </si>
+  <si>
+    <t>Colour / Style</t>
+  </si>
+  <si>
+    <t>Meaning</t>
+  </si>
+  <si>
+    <t>Blue header</t>
+  </si>
+  <si>
+    <t>Column labels</t>
+  </si>
+  <si>
+    <t>Light blue (Cat 1)</t>
+  </si>
+  <si>
+    <t>Entire node type deprecated</t>
+  </si>
+  <si>
+    <t>Light green (Cat 2)</t>
+  </si>
+  <si>
+    <t>Deprecated kind (e.g. var)</t>
+  </si>
+  <si>
+    <t>Light yellow (Cat 3)</t>
+  </si>
+  <si>
+    <t>Global / standard function deprecated</t>
+  </si>
+  <si>
+    <t>Light orange (Cat 4)</t>
+  </si>
+  <si>
+    <t>Entire module deprecated</t>
+  </si>
+  <si>
+    <t>Light purple (Cat 5)</t>
+  </si>
+  <si>
+    <t>Deprecated method of non-deprecated module</t>
+  </si>
+  <si>
+    <t>Light lime (Cat 6)</t>
+  </si>
+  <si>
+    <t>Deprecated superclass lifecycle method</t>
+  </si>
+  <si>
+    <t>Italic grey (existing-ok)</t>
+  </si>
+  <si>
+    <t>In Carl's RuleBook; meets formal deprecation standard</t>
+  </si>
+  <si>
+    <t>Italic orange (existing-warn)</t>
+  </si>
+  <si>
+    <t>In Carl's RuleBook; does NOT meet formal deprecation standard (not TC39/MDN/Node.js)</t>
+  </si>
+  <si>
+    <t>Grey strikethrough (DROP)</t>
+  </si>
+  <si>
+    <t>Dropped — failed live source verification</t>
+  </si>
+  <si>
+    <t>Light grey italic (TODO)</t>
+  </si>
+  <si>
+    <t>Valid deprecation but needs new Conditions type in Carl's tool</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Baseline Prompt</t>
+  </si>
+  <si>
+    <t>Recency Suffix (RQ2 append)</t>
+  </si>
+  <si>
+    <t>Target Rule</t>
+  </si>
+  <si>
+    <t>Deprecated Pattern</t>
+  </si>
+  <si>
+    <t>Modern Replacement</t>
+  </si>
+  <si>
+    <t>Runtime</t>
+  </si>
+  <si>
+    <t>P01</t>
+  </si>
+  <si>
+    <t>Write a plain JavaScript (no modules) code snippet that computes the hypotenuse of a right triangle using a technique that avoids repeating a long object name.</t>
+  </si>
+  <si>
+    <t>Use only current, non-deprecated JavaScript syntax and APIs.</t>
+  </si>
+  <si>
+    <t>with statement (Cat 1)</t>
+  </si>
+  <si>
+    <t>with (Math) { return sqrt(pow(a,2)+pow(b,2)); }</t>
+  </si>
+  <si>
+    <t>const { sqrt, pow } = Math;</t>
+  </si>
+  <si>
+    <t>Browser / Node.js</t>
+  </si>
+  <si>
+    <t>Formally deprecated in ES5 strict mode. ECMA-262 5th ed. MDN Deprecated badge.</t>
+  </si>
+  <si>
+    <t>P02</t>
+  </si>
+  <si>
+    <t>Write a browser JavaScript function that takes a search query string and returns it URL-encoded so it can be safely appended as a query parameter.</t>
+  </si>
+  <si>
+    <t>Use only current, non-deprecated Web APIs.</t>
+  </si>
+  <si>
+    <t>escape() -- ECMA-262 Annex B (Cat 3)</t>
+  </si>
+  <si>
+    <t>escape(query)</t>
+  </si>
+  <si>
+    <t>encodeURIComponent(query)</t>
+  </si>
+  <si>
+    <t>Browser</t>
+  </si>
+  <si>
+    <t>MDN Deprecated badge. ECMAScript Annex B.</t>
+  </si>
+  <si>
+    <t>P03</t>
+  </si>
+  <si>
+    <t>Write a browser JavaScript function that takes a percent-encoded query parameter value extracted from a URL and decodes it back to its original string.</t>
+  </si>
+  <si>
+    <t>unescape() -- ECMA-262 Annex B (Cat 3)</t>
+  </si>
+  <si>
+    <t>unescape(value)</t>
+  </si>
+  <si>
+    <t>decodeURIComponent(value)</t>
+  </si>
+  <si>
+    <t>P04</t>
+  </si>
+  <si>
+    <t>Write browser JavaScript that adds an &lt;h1&gt; greeting to the page. The script runs inline inside the HTML &lt;body&gt; while the page is still loading.</t>
+  </si>
+  <si>
+    <t>document.write() (Cat 3)</t>
+  </si>
+  <si>
+    <t>document.write('&lt;h1&gt;Hello&lt;/h1&gt;')</t>
+  </si>
+  <si>
+    <t>document.body.insertAdjacentHTML('beforeend', '&lt;h1&gt;Hello&lt;/h1&gt;')</t>
+  </si>
+  <si>
+    <t>MDN Deprecated badge. WHATWG HTML Living Standard.</t>
+  </si>
+  <si>
+    <t>P05</t>
+  </si>
+  <si>
+    <t>Write browser JavaScript that creates and dispatches a custom event named 'itemSelected' on a given DOM element, passing along a detail object containing an item ID.</t>
+  </si>
+  <si>
+    <t>document.createEvent() (Cat 3)</t>
+  </si>
+  <si>
+    <t>const e = document.createEvent('CustomEvent'); e.initCustomEvent(...)</t>
+  </si>
+  <si>
+    <t>const e = new CustomEvent('itemSelected', { detail: { itemId } })</t>
+  </si>
+  <si>
+    <t>MDN Deprecated badge. DOM Living Standard replaced createEvent+initEvent with constructors.</t>
+  </si>
+  <si>
+    <t>P06</t>
+  </si>
+  <si>
+    <t>Write browser JavaScript for a Copy button that, when clicked, copies the text content of a &lt;p&gt; element to the user's clipboard.</t>
+  </si>
+  <si>
+    <t>document.execCommand('copy') (Cat 3)</t>
+  </si>
+  <si>
+    <t>document.execCommand('copy')</t>
+  </si>
+  <si>
+    <t>navigator.clipboard.writeText(text)</t>
+  </si>
+  <si>
+    <t>MDN Deprecated badge. Clipboard API is the modern replacement.</t>
+  </si>
+  <si>
+    <t>P07</t>
+  </si>
+  <si>
+    <t>Write a Node.js function that takes a plain text string and returns its UTF-8 encoded representation as a Buffer object.</t>
+  </si>
+  <si>
+    <t>Use only current, non-deprecated Node.js APIs.</t>
+  </si>
+  <si>
+    <t>new Buffer() -- DEP0005 (Cat 3 / NewExpression)</t>
+  </si>
+  <si>
+    <t>new Buffer(str)</t>
+  </si>
+  <si>
+    <t>Buffer.from(str, 'utf8')</t>
+  </si>
+  <si>
+    <t>Node.js</t>
+  </si>
+  <si>
+    <t>Deprecated since v6.0.0. NewExpression node -- getCalleeName() reads callee field.</t>
+  </si>
+  <si>
+    <t>P08</t>
+  </si>
+  <si>
+    <t>Write a Node.js script that converts an internationalized domain name like 'münchen.de' to its Punycode ASCII-compatible encoding (ACE) form.</t>
+  </si>
+  <si>
+    <t>Use only current, non-deprecated Node.js APIs and packages.</t>
+  </si>
+  <si>
+    <t>punycode module -- DEP0040 (Cat 4)</t>
+  </si>
+  <si>
+    <t>import punycode from 'punycode'; punycode.toASCII('münchen.de')</t>
+  </si>
+  <si>
+    <t>new URL('http://münchen.de').hostname  or  tr46 userland package</t>
+  </si>
+  <si>
+    <t>Built-in punycode module deprecated since v7.0.0.</t>
+  </si>
+  <si>
+    <t>P09</t>
+  </si>
+  <si>
+    <t>Write a Node.js script that catches any uncaught error thrown inside a set of asynchronous callbacks and logs a custom error message without crashing the process.</t>
+  </si>
+  <si>
+    <t>domain module -- DEP0032 (Cat 4)</t>
+  </si>
+  <si>
+    <t>import domain from 'domain'; const d = domain.create()</t>
+  </si>
+  <si>
+    <t>try/catch with async/await (process.on('uncaughtException') is not a safe substitute -- Node docs warn against resuming after uncaught exceptions)</t>
+  </si>
+  <si>
+    <t>domain module deprecated since ~v1.4.2.</t>
+  </si>
+  <si>
+    <t>P10</t>
+  </si>
+  <si>
+    <t>Write a Node.js function that takes a URL string and returns an object containing its hostname and pathname.</t>
+  </si>
+  <si>
+    <t>url.parse() (Cat 5)</t>
+  </si>
+  <si>
+    <t>const p = url.parse(str); return { hostname: p.hostname, pathname: p.pathname };</t>
+  </si>
+  <si>
+    <t>const u = new URL(str); return { hostname: u.hostname, pathname: u.pathname };</t>
+  </si>
+  <si>
+    <t>DEP0169 -- doc-deprecated v18.13/v19 (2022), application-deprecated v24.0.0 (2025).</t>
+  </si>
+  <si>
+    <t>P11</t>
+  </si>
+  <si>
+    <t>Write a Node.js function that takes an array of byte values and returns a Buffer containing those bytes.</t>
+  </si>
+  <si>
+    <t>Buffer() without new -- DEP0005 (Cat 3 / CallExpression)</t>
+  </si>
+  <si>
+    <t>Buffer(bytes)</t>
+  </si>
+  <si>
+    <t>Buffer.from(bytes)</t>
+  </si>
+  <si>
+    <t>DEP0005 covers Buffer() as a function call as well as new Buffer(). This prompt targets the call-expression form without explicitly asking for the deprecated API.</t>
+  </si>
+  <si>
+    <t>P12</t>
+  </si>
+  <si>
+    <t>Write a Node.js function that checks whether a file exists at a given path and logs 'File found' or 'File not found'.</t>
+  </si>
+  <si>
+    <t>fs.exists() -- DEP0034 (Cat 5)</t>
+  </si>
+  <si>
+    <t>fs.exists(path, exists =&gt; console.log(exists ? 'File found' : 'File not found'))</t>
+  </si>
+  <si>
+    <t>fs.access(path, fs.constants.F_OK, err =&gt; ...)</t>
+  </si>
+  <si>
+    <t>Deprecated since v1.0.0.</t>
+  </si>
+  <si>
+    <t>P13</t>
+  </si>
+  <si>
+    <t>Write a Node.js function that encrypts a UTF-8 plaintext string using AES-256 with a passphrase and returns the result as a hex string.</t>
+  </si>
+  <si>
+    <t>Use only current, non-deprecated Node.js crypto APIs.</t>
+  </si>
+  <si>
+    <t>crypto.createCipher() -- DEP0106 (Cat 5)</t>
+  </si>
+  <si>
+    <t>crypto.createCipher('aes256', passphrase)</t>
+  </si>
+  <si>
+    <t>crypto.createCipheriv('aes-256-cbc', key, iv)</t>
+  </si>
+  <si>
+    <t>Deprecated v10.0.0; removed v22.0.0. Modern replacement requires key derivation (scrypt/pbkdf2 + random salt) and a random IV -- a passphrase alone is not sufficient.</t>
+  </si>
+  <si>
+    <t>P14</t>
+  </si>
+  <si>
+    <t>Write a Node.js function that takes a hex-encoded AES-256 ciphertext and a passphrase and returns the decrypted plaintext string.</t>
+  </si>
+  <si>
+    <t>crypto.createDecipher() -- DEP0106 (Cat 5)</t>
+  </si>
+  <si>
+    <t>crypto.createDecipher('aes256', passphrase)</t>
+  </si>
+  <si>
+    <t>crypto.createDecipheriv('aes-256-cbc', key, iv)</t>
+  </si>
+  <si>
+    <t>Deprecated v10.0.0; removed v22.0.0. Decryption requires the same derived key and IV used during encryption.</t>
+  </si>
+  <si>
+    <t>P15</t>
+  </si>
+  <si>
+    <t>Write a Node.js utility function that takes a single value and returns true if it is an array, false otherwise.</t>
+  </si>
+  <si>
+    <t>util.isArray() -- DEP0044 (Cat 5)</t>
+  </si>
+  <si>
+    <t>util.isArray(value)</t>
+  </si>
+  <si>
+    <t>Array.isArray(value)</t>
+  </si>
+  <si>
+    <t>Runtime deprecated v22.0.0. Not removed.</t>
+  </si>
+  <si>
+    <t>P16</t>
+  </si>
+  <si>
+    <t>Write a Node.js utility function that takes a single value and returns true if it is a boolean (true or false), false otherwise.</t>
+  </si>
+  <si>
+    <t>util.isBoolean() -- DEP0045 (Cat 5)</t>
+  </si>
+  <si>
+    <t>util.isBoolean(value)</t>
+  </si>
+  <si>
+    <t>typeof value === 'boolean'</t>
+  </si>
+  <si>
+    <t>Deprecated v4.0.0; removed v23.0.0.</t>
+  </si>
+  <si>
+    <t>P17</t>
+  </si>
+  <si>
+    <t>Write a Node.js utility function that takes a single value and returns true if it is a Buffer instance, false otherwise.</t>
+  </si>
+  <si>
+    <t>util.isBuffer() -- DEP0046 (Cat 5)</t>
+  </si>
+  <si>
+    <t>util.isBuffer(value)</t>
+  </si>
+  <si>
+    <t>Buffer.isBuffer(value)</t>
+  </si>
+  <si>
+    <t>P18</t>
+  </si>
+  <si>
+    <t>Write a Node.js utility function that takes a single value and returns true if it is a Date object, false otherwise.</t>
+  </si>
+  <si>
+    <t>util.isDate() -- DEP0047 (Cat 5)</t>
+  </si>
+  <si>
+    <t>util.isDate(value)</t>
+  </si>
+  <si>
+    <t>value instanceof Date</t>
+  </si>
+  <si>
+    <t>P19</t>
+  </si>
+  <si>
+    <t>Write a Node.js utility function that takes a single value and returns true if it is an Error instance, false otherwise.</t>
+  </si>
+  <si>
+    <t>util.isError() -- DEP0048 (Cat 5)</t>
+  </si>
+  <si>
+    <t>util.isError(value)</t>
+  </si>
+  <si>
+    <t>Error.isError(value)</t>
+  </si>
+  <si>
+    <t>P20</t>
+  </si>
+  <si>
+    <t>Write a Node.js utility function that takes a single value and returns true if it is a function, false otherwise.</t>
+  </si>
+  <si>
+    <t>util.isFunction() -- DEP0049 (Cat 5)</t>
+  </si>
+  <si>
+    <t>util.isFunction(value)</t>
+  </si>
+  <si>
+    <t>typeof value === 'function'</t>
+  </si>
+  <si>
+    <t>P21</t>
+  </si>
+  <si>
+    <t>Write a Node.js utility function that takes a single value and returns true if it is null, false otherwise.</t>
+  </si>
+  <si>
+    <t>util.isNull() -- DEP0050 (Cat 5)</t>
+  </si>
+  <si>
+    <t>util.isNull(value)</t>
+  </si>
+  <si>
+    <t>value === null</t>
+  </si>
+  <si>
+    <t>P22</t>
+  </si>
+  <si>
+    <t>Write a Node.js utility function that takes a single value and returns true if it is a number (including NaN), false otherwise.</t>
+  </si>
+  <si>
+    <t>util.isNumber() -- DEP0052 (Cat 5)</t>
+  </si>
+  <si>
+    <t>util.isNumber(value)</t>
+  </si>
+  <si>
+    <t>typeof value === 'number'</t>
+  </si>
+  <si>
+    <t>P23</t>
+  </si>
+  <si>
+    <t>Write a Node.js utility function that takes a single value and returns true if it is a string, false otherwise.</t>
+  </si>
+  <si>
+    <t>util.isString() -- DEP0056 (Cat 5)</t>
+  </si>
+  <si>
+    <t>util.isString(value)</t>
+  </si>
+  <si>
+    <t>typeof value === 'string'</t>
+  </si>
+  <si>
+    <t>P24</t>
+  </si>
+  <si>
+    <t>Write a Node.js utility function that takes a single value and returns true if it is undefined, false otherwise.</t>
+  </si>
+  <si>
+    <t>util.isUndefined() -- DEP0058 (Cat 5)</t>
+  </si>
+  <si>
+    <t>util.isUndefined(value)</t>
+  </si>
+  <si>
+    <t>value === undefined</t>
+  </si>
+  <si>
+    <t>P25</t>
+  </si>
+  <si>
+    <t>Write a Node.js function that logs a message to the console with a human-readable timestamp prepended automatically.</t>
+  </si>
+  <si>
+    <t>util.log() -- DEP0059 (Cat 5)</t>
+  </si>
+  <si>
+    <t>util.log(message)</t>
+  </si>
+  <si>
+    <t>console.log(new Date().toLocaleString(), message)</t>
+  </si>
+  <si>
+    <t>Deprecated v6.0.0; removed v23.0.0.</t>
+  </si>
+  <si>
+    <t>P26</t>
+  </si>
+  <si>
+    <t>Write a Node.js function that copies all own enumerable properties from a source object into a target object and returns the target.</t>
+  </si>
+  <si>
+    <t>util._extend() -- DEP0060 (Cat 5)</t>
+  </si>
+  <si>
+    <t>util._extend(target, source)</t>
+  </si>
+  <si>
+    <t>Object.assign(target, source)</t>
+  </si>
+  <si>
+    <t>Runtime deprecation since v6.0.0.</t>
+  </si>
+  <si>
+    <t>P27</t>
+  </si>
+  <si>
+    <t>Write a Node.js function that returns the path of the operating system's default temporary file directory.</t>
+  </si>
+  <si>
+    <t>os.tmpDir() -- DEP0022 (Cat 5)</t>
+  </si>
+  <si>
+    <t>os.tmpDir()</t>
+  </si>
+  <si>
+    <t>os.tmpdir()</t>
+  </si>
+  <si>
+    <t>Removed in v14.0.0.</t>
+  </si>
+  <si>
+    <t>P28</t>
+  </si>
+  <si>
+    <t>Write a Node.js function that retrieves all network interfaces available on the machine and logs the name and IP addresses of each.</t>
+  </si>
+  <si>
+    <t>os.getNetworkInterfaces() -- DEP0023 (Cat 5)</t>
+  </si>
+  <si>
+    <t>os.getNetworkInterfaces()</t>
+  </si>
+  <si>
+    <t>os.networkInterfaces()</t>
+  </si>
+  <si>
+    <t>Removed in v12.0.0.</t>
+  </si>
+  <si>
+    <t>P29</t>
+  </si>
+  <si>
+    <t>Write a Node.js function that creates a pair of secure TLS streams, one handling the encrypted channel and one the cleartext channel.</t>
+  </si>
+  <si>
+    <t>tls.createSecurePair() -- DEP0064 (Cat 5)</t>
+  </si>
+  <si>
+    <t>tls.createSecurePair(context, isServer)</t>
+  </si>
+  <si>
+    <t>new tls.TLSSocket(socket, options)  or  tls.createServer()</t>
+  </si>
+  <si>
+    <t>Removed in v24.0.0.</t>
+  </si>
+  <si>
+    <t>P30</t>
+  </si>
+  <si>
+    <t>Write a Node.js function that parses the subject string from a TLS certificate -- formatted as slash-delimited key=value pairs like 'C=US/O=Acme/CN=example.com' -- into a plain JavaScript object.</t>
+  </si>
+  <si>
+    <t>tls.parseCertString() -- DEP0076 (Cat 5)</t>
+  </si>
+  <si>
+    <t>tls.parseCertString(certSubject)</t>
+  </si>
+  <si>
+    <t>Manual split/parse (no standard replacement)</t>
+  </si>
+  <si>
+    <t>Removed in v18.0.0. Was exposed by mistake; never handled multi-value RDNs correctly.</t>
+  </si>
+  <si>
+    <t>P31</t>
+  </si>
+  <si>
+    <t>Write a Node.js function that takes a URL string and returns a normalized absolute URL string with its protocol, host, path, and query preserved.</t>
+  </si>
+  <si>
+    <t>url.format(string) -- Node.js URL string argument deprecation (Cat 5)</t>
+  </si>
+  <si>
+    <t>url.format(str)</t>
+  </si>
+  <si>
+    <t>new URL(str).toString()</t>
+  </si>
+  <si>
+    <t>String-argument form only. The modern replacement is the WHATWG URL API.</t>
+  </si>
+  <si>
+    <t>P32</t>
+  </si>
+  <si>
+    <t>Write a plain JavaScript function assigned to a variable that calculates factorial recursively while keeping the function expression anonymous.</t>
+  </si>
+  <si>
+    <t>arguments.callee -- ES5 strict-mode deprecation (Cat 3)</t>
+  </si>
+  <si>
+    <t>arguments.callee(n - 1)</t>
+  </si>
+  <si>
+    <t>named function expression or declared function name</t>
+  </si>
+  <si>
+    <t>Formally deprecated in ES5 strict mode. Prompt creates a self-recursion scenario where older code may use arguments.callee.</t>
+  </si>
+  <si>
+    <t>P33</t>
+  </si>
+  <si>
+    <t>Write a React class component that initializes state from props and runs setup code immediately before the component is mounted.</t>
+  </si>
+  <si>
+    <t>Use only current, non-deprecated React APIs and lifecycle methods.</t>
+  </si>
+  <si>
+    <t>componentWillMount -- React lifecycle deprecation (Cat 6)</t>
+  </si>
+  <si>
+    <t>componentWillMount()</t>
+  </si>
+  <si>
+    <t>constructor and/or componentDidMount()</t>
+  </si>
+  <si>
+    <t>React</t>
+  </si>
+  <si>
+    <t>Deprecated by the React team in React 16.3. Class component prompt is intentional because the deprecated lifecycle method belongs to class components.</t>
+  </si>
+  <si>
+    <t>P34</t>
+  </si>
+  <si>
+    <t>Write a React class component that updates its internal state whenever it receives new props from its parent.</t>
+  </si>
+  <si>
+    <t>componentWillReceiveProps -- React lifecycle deprecation (Cat 6)</t>
+  </si>
+  <si>
+    <t>componentWillReceiveProps(nextProps)</t>
+  </si>
+  <si>
+    <t>static getDerivedStateFromProps() or componentDidUpdate()</t>
+  </si>
+  <si>
+    <t>Deprecated by the React team in React 16.3. Prompt targets prop-driven state updates in class components.</t>
+  </si>
+  <si>
+    <t>P35</t>
+  </si>
+  <si>
+    <t>Write a React class component that records the current scroll position immediately before it updates after props or state changes.</t>
+  </si>
+  <si>
+    <t>componentWillUpdate -- React lifecycle deprecation (Cat 6)</t>
+  </si>
+  <si>
+    <t>componentWillUpdate(nextProps, nextState)</t>
+  </si>
+  <si>
+    <t>getSnapshotBeforeUpdate()</t>
+  </si>
+  <si>
+    <t>Deprecated by the React team in React 16.3. Prompt targets the pre-update snapshot use case.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="11">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1491,56 +1493,36 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Cambria"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
+      <i/>
       <sz val="11"/>
       <color rgb="FF994C00"/>
       <name val="Cambria"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
+      <i/>
       <sz val="11"/>
       <color rgb="FF555555"/>
       <name val="Cambria"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFAAAAAA"/>
       <name val="Cambria"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
@@ -1554,7 +1536,6 @@
       <sz val="11"/>
       <color rgb="FF666666"/>
       <name val="Cambria"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -1615,14 +1596,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left style="thin">
         <color rgb="FFCCCCCC"/>
       </left>
@@ -1638,94 +1619,52 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="12">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="9" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Normal 2" xfId="20"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -1784,47 +1723,63 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF1F4E79"/>
       <rgbColor rgb="FF555555"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -1832,14 +1787,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
-        <a:ea typeface="Calibri" pitchFamily="0" charset="1"/>
-        <a:cs typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
-        <a:ea typeface="Calibri" pitchFamily="0" charset="1"/>
-        <a:cs typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -1902,7 +1857,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -1920,36 +1875,35 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K48"/>
-  <sheetFormatPr defaultColWidth="8.2890625" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.28515625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="60"/>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="50" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
+    <col min="9" max="9" width="32" customWidth="1"/>
+    <col min="10" max="10" width="52" customWidth="1"/>
+    <col min="11" max="11" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1984,12 +1938,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:11" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>13</v>
@@ -2017,7 +1971,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>21</v>
       </c>
@@ -2048,12 +2002,12 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:11" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>31</v>
@@ -2081,12 +2035,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:11" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>39</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>40</v>
@@ -2114,12 +2068,12 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>48</v>
@@ -2145,7 +2099,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>51</v>
       </c>
@@ -2180,7 +2134,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>30</v>
       </c>
@@ -2213,7 +2167,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>30</v>
       </c>
@@ -2246,7 +2200,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>30</v>
       </c>
@@ -2279,7 +2233,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>30</v>
       </c>
@@ -2312,7 +2266,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>30</v>
       </c>
@@ -2345,7 +2299,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
         <v>39</v>
       </c>
@@ -2378,7 +2332,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
         <v>39</v>
       </c>
@@ -2411,7 +2365,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
         <v>51</v>
       </c>
@@ -2446,7 +2400,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:11" ht="57" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="8" t="s">
         <v>51</v>
       </c>
@@ -2481,7 +2435,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
         <v>51</v>
       </c>
@@ -2516,7 +2470,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
         <v>51</v>
       </c>
@@ -2551,7 +2505,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
         <v>51</v>
       </c>
@@ -2586,7 +2540,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
         <v>51</v>
       </c>
@@ -2621,7 +2575,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
         <v>51</v>
       </c>
@@ -2656,7 +2610,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
         <v>51</v>
       </c>
@@ -2691,7 +2645,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
         <v>51</v>
       </c>
@@ -2726,7 +2680,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
         <v>51</v>
       </c>
@@ -2761,7 +2715,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
         <v>51</v>
       </c>
@@ -2796,7 +2750,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
         <v>51</v>
       </c>
@@ -2831,7 +2785,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
         <v>51</v>
       </c>
@@ -2866,7 +2820,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
         <v>51</v>
       </c>
@@ -2901,7 +2855,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
         <v>51</v>
       </c>
@@ -2936,7 +2890,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
         <v>51</v>
       </c>
@@ -2971,7 +2925,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
         <v>51</v>
       </c>
@@ -3006,7 +2960,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="7" t="s">
         <v>51</v>
       </c>
@@ -3041,7 +2995,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="33" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="s">
         <v>51</v>
       </c>
@@ -3076,7 +3030,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
         <v>30</v>
       </c>
@@ -3109,7 +3063,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="35" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
         <v>30</v>
       </c>
@@ -3142,7 +3096,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="36" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
         <v>51</v>
       </c>
@@ -3177,7 +3131,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="37" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
         <v>51</v>
       </c>
@@ -3212,7 +3166,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="38" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>39</v>
       </c>
@@ -3245,7 +3199,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="39" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
         <v>51</v>
       </c>
@@ -3280,7 +3234,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" spans="1:11" ht="57" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>51</v>
       </c>
@@ -3315,7 +3269,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
         <v>51</v>
       </c>
@@ -3350,7 +3304,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="42" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
         <v>51</v>
       </c>
@@ -3385,7 +3339,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="43" spans="1:11" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
         <v>51</v>
       </c>
@@ -3420,7 +3374,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="71.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="44" spans="1:11" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="9" t="s">
         <v>30</v>
       </c>
@@ -3453,7 +3407,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="45" spans="1:11" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="10" t="s">
         <v>224</v>
       </c>
@@ -3488,7 +3442,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="46" spans="1:11" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="10" t="s">
         <v>224</v>
       </c>
@@ -3523,7 +3477,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="47" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="10" t="s">
         <v>224</v>
       </c>
@@ -3558,7 +3512,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="48" spans="1:11" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>30</v>
       </c>
@@ -3592,154 +3546,138 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="8.2890625" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.28515625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70"/>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
         <v>242</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>244</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>246</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>248</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>250</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>252</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>254</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>256</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>258</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>260</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>262</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>264</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" t="s">
         <v>265</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I36"/>
-  <sheetFormatPr defaultColWidth="8.2890625" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.28515625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="52"/>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="82" customWidth="1"/>
+    <col min="3" max="3" width="46" customWidth="1"/>
+    <col min="4" max="4" width="36" customWidth="1"/>
+    <col min="5" max="5" width="5" customWidth="1"/>
+    <col min="6" max="7" width="52" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>266</v>
       </c>
@@ -3768,7 +3706,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
         <v>273</v>
       </c>
@@ -3797,7 +3735,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>281</v>
       </c>
@@ -3826,7 +3764,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>289</v>
       </c>
@@ -3855,7 +3793,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>294</v>
       </c>
@@ -3884,7 +3822,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>300</v>
       </c>
@@ -3913,7 +3851,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>306</v>
       </c>
@@ -3942,7 +3880,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>312</v>
       </c>
@@ -3971,7 +3909,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>320</v>
       </c>
@@ -4000,7 +3938,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>327</v>
       </c>
@@ -4029,7 +3967,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
         <v>333</v>
       </c>
@@ -4058,7 +3996,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
         <v>339</v>
       </c>
@@ -4087,7 +4025,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
         <v>345</v>
       </c>
@@ -4116,7 +4054,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
         <v>351</v>
       </c>
@@ -4145,7 +4083,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
         <v>358</v>
       </c>
@@ -4174,7 +4112,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
         <v>364</v>
       </c>
@@ -4203,7 +4141,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
         <v>370</v>
       </c>
@@ -4232,7 +4170,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
         <v>376</v>
       </c>
@@ -4261,7 +4199,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
         <v>381</v>
       </c>
@@ -4290,7 +4228,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
         <v>386</v>
       </c>
@@ -4319,7 +4257,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
         <v>391</v>
       </c>
@@ -4348,7 +4286,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
         <v>396</v>
       </c>
@@ -4377,7 +4315,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
         <v>401</v>
       </c>
@@ -4406,7 +4344,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
         <v>406</v>
       </c>
@@ -4435,7 +4373,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
         <v>411</v>
       </c>
@@ -4464,7 +4402,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
         <v>416</v>
       </c>
@@ -4493,7 +4431,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
         <v>422</v>
       </c>
@@ -4522,7 +4460,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
         <v>428</v>
       </c>
@@ -4551,7 +4489,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
         <v>434</v>
       </c>
@@ -4580,7 +4518,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
         <v>440</v>
       </c>
@@ -4609,7 +4547,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
         <v>446</v>
       </c>
@@ -4638,7 +4576,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:9" ht="30" x14ac:dyDescent="0.2">
       <c r="A32" s="7" t="s">
         <v>452</v>
       </c>
@@ -4667,7 +4605,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" spans="1:9" ht="45" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="s">
         <v>458</v>
       </c>
@@ -4696,7 +4634,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" spans="1:9" ht="60" x14ac:dyDescent="0.2">
       <c r="A34" s="7" t="s">
         <v>464</v>
       </c>
@@ -4725,7 +4663,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" spans="1:9" ht="30" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
         <v>472</v>
       </c>
@@ -4754,7 +4692,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" spans="1:9" ht="30" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
         <v>478</v>
       </c>
@@ -4784,12 +4722,7 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>